<commit_message>
feat(viceri-study): publish specification and test suite v1.6
</commit_message>
<xml_diff>
--- a/output/xlsx/AdministradorAdicionaCompatibilidade--GT-.xlsx
+++ b/output/xlsx/AdministradorAdicionaCompatibilidade--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="49">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 6 test case(s)</t>
+    <t>Size: 4 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -122,52 +122,34 @@
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Volta para listagem de Compatibilidades</t>
-  </si>
-  <si>
-    <t>Administrador: clica no botao Voltar</t>
+    <t>Exception Flow 1: Nao insere algum dado obrigatorio'</t>
+  </si>
+  <si>
+    <t>SYSTEM informa que os dados obrigatorios devem ser preenchidos</t>
+  </si>
+  <si>
+    <t>Administrador: preenche dados obrigatorios e clica em Atualizar</t>
+  </si>
+  <si>
+    <t>SYSTEM processes action successfully</t>
+  </si>
+  <si>
+    <t>Flow interrupted due to exception / error</t>
   </si>
   <si>
     <t>TC3</t>
   </si>
   <si>
-    <t>Alternative Flow 2: Cancelar registro de nova Compatibilidade</t>
-  </si>
-  <si>
-    <t>Administrador: clica no botao Cancelar</t>
+    <t>Exception Flow 2: Usuario insere Tipo de Mercadoria invalido</t>
+  </si>
+  <si>
+    <t>SYSTEM alerta que Tipo de Mercadoria e invalido</t>
+  </si>
+  <si>
+    <t>Administrador: preenche um Tipo de Mercadoria valido e clica em Atualizar</t>
   </si>
   <si>
     <t>TC4</t>
-  </si>
-  <si>
-    <t>Exception Flow 1: Nao insere algum dado obrigatorio'</t>
-  </si>
-  <si>
-    <t>SYSTEM informa que os dados obrigatorios devem ser preenchidos</t>
-  </si>
-  <si>
-    <t>Administrador: preenche dados obrigatorios e clica em Atualizar</t>
-  </si>
-  <si>
-    <t>SYSTEM processes action successfully</t>
-  </si>
-  <si>
-    <t>Flow interrupted due to exception / error</t>
-  </si>
-  <si>
-    <t>TC5</t>
-  </si>
-  <si>
-    <t>Exception Flow 2: Usuario insere Tipo de Mercadoria invalido</t>
-  </si>
-  <si>
-    <t>SYSTEM alerta que Tipo de Mercadoria e invalido</t>
-  </si>
-  <si>
-    <t>Administrador: preenche um Tipo de Mercadoria valido e clica em Atualizar</t>
-  </si>
-  <si>
-    <t>TC6</t>
   </si>
   <si>
     <t>Exception Flow 3: Usuario insere NCM invalido</t>
@@ -268,7 +250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
@@ -517,13 +499,13 @@
         <v>2.0</v>
       </c>
       <c r="B21" t="s" s="3">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D21" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E21" t="s" s="3">
         <v>27</v>
@@ -537,13 +519,13 @@
         <v>3.0</v>
       </c>
       <c r="B22" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D22" t="s" s="3">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s" s="3">
         <v>27</v>
@@ -557,13 +539,13 @@
         <v>4.0</v>
       </c>
       <c r="B23" t="s" s="3">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D23" t="s" s="3">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E23" t="s" s="3">
         <v>27</v>
@@ -577,7 +559,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27">
@@ -585,7 +567,7 @@
         <v>11</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s" s="1">
         <v>13</v>
@@ -599,7 +581,7 @@
         <v>15</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E28" t="s" s="1">
         <v>17</v>
@@ -678,13 +660,13 @@
         <v>3.0</v>
       </c>
       <c r="B33" t="s" s="3">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C33" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D33" t="s" s="3">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="E33" t="s" s="3">
         <v>27</v>
@@ -698,13 +680,13 @@
         <v>4.0</v>
       </c>
       <c r="B34" t="s" s="3">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C34" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D34" t="s" s="3">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E34" t="s" s="3">
         <v>27</v>
@@ -714,98 +696,98 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B35" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C35" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D35" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="E35" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F35" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s" s="1">
+      <c r="A35" t="s" s="1">
         <v>33</v>
       </c>
-      <c r="B36" t="s" s="0">
-        <v>34</v>
+      <c r="B35" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>41</v>
-      </c>
-      <c r="C39" t="s" s="1">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E39" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="E40" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B41" t="s" s="0">
-        <v>19</v>
+      <c r="A41" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D41" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E41" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F41" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B42" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C42" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D42" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E42" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F42" t="s" s="2">
-        <v>25</v>
+      <c r="A42" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B42" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C42" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D42" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E42" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F42" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B43" t="s" s="3">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C43" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D43" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E43" t="s" s="3">
         <v>27</v>
@@ -816,16 +798,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B44" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C44" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D44" t="s" s="3">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="E44" t="s" s="3">
         <v>27</v>
@@ -836,16 +818,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B45" t="s" s="3">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C45" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D45" t="s" s="3">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E45" t="s" s="3">
         <v>27</v>
@@ -855,313 +837,11 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B46" t="s" s="3">
-        <v>44</v>
-      </c>
-      <c r="C46" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D46" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="E46" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F46" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="s" s="1">
+      <c r="A46" t="s" s="1">
         <v>33</v>
       </c>
-      <c r="B47" t="s" s="0">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B50" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="C50" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E50" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B51" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="E51" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B52" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C53" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D53" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E53" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F53" t="s" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B54" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C54" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D54" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E54" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F54" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B55" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C55" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D55" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="E55" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F55" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B56" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C56" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D56" t="s" s="3">
-        <v>49</v>
-      </c>
-      <c r="E56" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F56" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B57" t="s" s="3">
-        <v>50</v>
-      </c>
-      <c r="C57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D57" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="E57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F57" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s" s="1">
-        <v>33</v>
-      </c>
-      <c r="B58" t="s" s="0">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B61" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="C61" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E61" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B62" t="s" s="0">
-        <v>52</v>
-      </c>
-      <c r="E62" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B63" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B64" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C64" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D64" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E64" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F64" t="s" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B65" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C65" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D65" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E65" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F65" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B66" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C66" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D66" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="E66" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F66" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B67" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C67" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D67" t="s" s="3">
-        <v>53</v>
-      </c>
-      <c r="E67" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F67" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B68" t="s" s="3">
-        <v>54</v>
-      </c>
-      <c r="C68" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D68" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="E68" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F68" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="s" s="1">
-        <v>33</v>
-      </c>
-      <c r="B69" t="s" s="0">
-        <v>46</v>
+      <c r="B46" t="s" s="0">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>